<commit_message>
Remove o Kit Camping 6 itens e troca o destaque da home
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/links.xlsx
+++ b/data/links.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -523,24 +523,24 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Kit Legendários Camping Acampamento 6 Itens Barraca Completo (Barraca, Lona, Saco de Dormir, Isolante Termico, Poncho impermeável, Lanterna de cabeça)</t>
+          <t>New Hawaii Barraca Camping Automática 2 Pessoas 1200mm Impermeável Upf50+</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Kit</t>
+          <t>Barraca</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://meli.la/1LaRLiq</t>
+          <t>https://meli.la/19US1iZ</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>New Hawaii Barraca Camping Automática 2 Pessoas 1200mm Impermeável Upf50+</t>
+          <t>Barraca Joyfox Para 2 Pessoas, Impermeável 3500mm e Ultraleve</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -550,14 +550,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://meli.la/19US1iZ</t>
+          <t>https://meli.la/13MSwEB</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Barraca Joyfox Para 2 Pessoas, Impermeável 3500mm e Ultraleve</t>
+          <t>Barraca Camping Windy 1 Pessoa Ntk Acampamento Impermeável Cor Laranja</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -567,31 +567,31 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://meli.la/13MSwEB</t>
+          <t>https://meli.la/1eHU6qb</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Barraca Camping Windy 1 Pessoa Ntk Acampamento Impermeável Cor Laranja</t>
+          <t>Cobertor Fleece De Camping - Cor Cinza</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Barraca</t>
+          <t>Cobertor</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://meli.la/1eHU6qb</t>
+          <t>https://meli.la/1AH1BAm</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cobertor Fleece De Camping - Cor Cinza</t>
+          <t>Coberta Manta Soft Solteiro Microfibra Anti-alérgica</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -601,31 +601,31 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://meli.la/1AH1BAm</t>
+          <t>https://meli.la/2dpniX9</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Coberta Manta Soft Solteiro Microfibra Anti-alérgica</t>
+          <t>Colchão Inflável Solteiro Com Bomba Inflador Camping Viagem</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cobertor</t>
+          <t>Colchão</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://meli.la/2dpniX9</t>
+          <t>https://meli.la/1vtyiAL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Colchão Inflável Solteiro Com Bomba Inflador Camping Viagem</t>
+          <t>Colchonete Inflável Solteiro Joyfox 190x60cm Verde Com Travesseiro e Bomba Manual</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -635,14 +635,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://meli.la/1vtyiAL</t>
+          <t>https://meli.la/1qTvrq9</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Colchonete Inflável Solteiro Joyfox 190x60cm Verde Com Travesseiro e Bomba Manual</t>
+          <t>Colchão Inflável Solteiro De Luxo Com Bomba Recarregável Portátil Integrada, Completo Com Almofada E Bolsa De Armazenamento Joyfox</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -652,31 +652,31 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://meli.la/1qTvrq9</t>
+          <t>https://meli.la/1Fg86tw</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Colchão Inflável Solteiro De Luxo Com Bomba Recarregável Portátil Integrada, Completo Com Almofada E Bolsa De Armazenamento Joyfox</t>
+          <t>Isolante Tapete Térmico Em Eva Para Camping Aluminizado</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Colchão</t>
+          <t>Isolante Térmico</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://meli.la/1Fg86tw</t>
+          <t>https://meli.la/1Ag26Jd</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Isolante Tapete Térmico Em Eva Para Camping Aluminizado</t>
+          <t>Isolante Térmico Dobrável Naturehike Egg Crate R.value 1.8</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -686,14 +686,14 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://meli.la/1Ag26Jd</t>
+          <t>https://meli.la/1Kqts5D</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Isolante Térmico Dobrável Naturehike Egg Crate R.value 1.8</t>
+          <t>Isolante Termico Dobravel Solteiro 180x50 Thor Azteq Xpe 8mm</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -703,31 +703,31 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://meli.la/1Kqts5D</t>
+          <t>https://meli.la/1Lzrc7W</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Isolante Termico Dobravel Solteiro 180x50 Thor Azteq Xpe 8mm</t>
+          <t>Camplivre Mochila De Hidratação Ataque 20l Camping Trilha</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Isolante Térmico</t>
+          <t>Mochila de Ataque</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://meli.la/1Lzrc7W</t>
+          <t>https://meli.la/2uqzD7a</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Camplivre Mochila De Hidratação Ataque 20l Camping Trilha</t>
+          <t>Mochila Ntk Attack Air X 30 Litros Laranja (Compativel com bolsa de água vendida separadamente)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -737,14 +737,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://meli.la/2uqzD7a</t>
+          <t>https://meli.la/24nVLeH</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mochila Ntk Attack Air X 30 Litros Laranja (Compativel com bolsa de água vendida separadamente)</t>
+          <t>Mochila De Hidratação Bolsa De Agua 3 Litros Com Refil Incluso Bike Ciclismo Acampamento Corrida Trilha Caminhada Tumblr Cor Verde-escuro</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -754,48 +754,48 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://meli.la/24nVLeH</t>
+          <t>https://meli.la/1GKpT9v</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mochila De Hidratação Bolsa De Agua 3 Litros Com Refil Incluso Bike Ciclismo Acampamento Corrida Trilha Caminhada Tumblr Cor Verde-escuro</t>
+          <t>Refil Reservatório De Água 2l P/ Mochila Hidratação</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Mochila de Ataque</t>
+          <t>Refil de água</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://meli.la/1GKpT9v</t>
+          <t>https://meli.la/2A3aaDY</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Refil Reservatório De Água 2l P/ Mochila Hidratação</t>
+          <t>Bastão De Caminhada Nautika Retrátil Sistema Anti-shock</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Refil de água</t>
+          <t>Bastão de caminhada</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://meli.la/2A3aaDY</t>
+          <t>https://meli.la/1j6taRn</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Bastão De Caminhada Nautika Retrátil Sistema Anti-shock</t>
+          <t>Bastão De Caminhada Dobrável Antiderrapante Cajado Trekking</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -805,14 +805,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://meli.la/1j6taRn</t>
+          <t>https://meli.la/1ubUqAr</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bastão De Caminhada Dobrável Antiderrapante Cajado Trekking</t>
+          <t>Cajado Madeira Legendário 160cm - Personlizado</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -822,31 +822,31 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://meli.la/1ubUqAr</t>
+          <t>https://meli.la/2zzHKBM</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Cajado Madeira Legendário 160cm - Personlizado</t>
+          <t>Lanterna Cabeça Led Headlamp 140 Lumens Luz Vermelha Branca</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Bastão de caminhada</t>
+          <t>Lanterna de cabeça</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://meli.la/2zzHKBM</t>
+          <t>https://meli.la/2QND6hg</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Lanterna Cabeça Led Headlamp 140 Lumens Luz Vermelha Branca</t>
+          <t>Lanterna De Boné / Cabeça Nitecore Nu11 150 Lumens C/sensor</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -856,14 +856,14 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://meli.la/2QND6hg</t>
+          <t>https://meli.la/2tXPbeb</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Lanterna De Boné / Cabeça Nitecore Nu11 150 Lumens C/sensor</t>
+          <t>Lanterna Recarregável Led Boné Pescaria Ajustável Ciclismo</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -873,48 +873,48 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://meli.la/2tXPbeb</t>
+          <t>https://meli.la/1mhrDp9</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Lanterna Recarregável Led Boné Pescaria Ajustável Ciclismo</t>
+          <t>Lona 2x2 Azul Impermeavel Piscina Barraca Camping Telhado</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Lanterna de cabeça</t>
+          <t>Lona</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://meli.la/1mhrDp9</t>
+          <t>https://meli.la/335cE5E</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Lona 2x2 Azul Impermeavel Piscina Barraca Camping Telhado</t>
+          <t>Saco De Dormir Camping Impermeável Usd Confortável 2,10m X 75cm C/ Bolsa De Transporte</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Lona</t>
+          <t>Saco de dormir</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://meli.la/335cE5E</t>
+          <t>https://meli.la/2XKrnfN</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Saco De Dormir Camping Impermeável Usd Confortável 2,10m X 75cm C/ Bolsa De Transporte</t>
+          <t>Joyfox Saco De Dormir Com Zíper Duplo E Abertura Para Os Braços 210 x 75 cm Verde Conforto, Impermeável E Portátil Para Camping</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -924,14 +924,14 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://meli.la/2XKrnfN</t>
+          <t>https://meli.la/2kVYYwi</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Joyfox Saco De Dormir Com Zíper Duplo E Abertura Para Os Braços 210 x 75 cm Verde Conforto, Impermeável E Portátil Para Camping</t>
+          <t>Saco De Dormir Ntk Viper Legendários Conforto Em Aventuras Laranja</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -941,31 +941,31 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://meli.la/2kVYYwi</t>
+          <t>https://meli.la/2TPVvHF</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Saco De Dormir Ntk Viper Legendários Conforto Em Aventuras Laranja</t>
+          <t>Travesseiro Inflável Para Camping Leve E Dobrável Conforto</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Saco de dormir</t>
+          <t>Travesseiro</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://meli.la/2TPVvHF</t>
+          <t>https://meli.la/181N8Cc</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Travesseiro Inflável Para Camping Leve E Dobrável Conforto</t>
+          <t>Travesseiro Inflável Camping Viagem Carro Praia Prova D'água</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -975,31 +975,31 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://meli.la/181N8Cc</t>
+          <t>https://meli.la/2w1JZp7</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Travesseiro Inflável Camping Viagem Carro Praia Prova D'água</t>
+          <t>Tênis Para Legendários Fila Racer Skytrail Masculino</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Travesseiro</t>
+          <t>Tenis</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://meli.la/2w1JZp7</t>
+          <t>https://meli.la/2nYMff7</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Tênis Para Legendários Fila Racer Skytrail Masculino</t>
+          <t>Tênis Asics Trabuco Terra 3 Preto E Laranja</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1009,14 +1009,14 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://meli.la/2nYMff7</t>
+          <t>https://meli.la/2sL3u8E</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Tênis Asics Trabuco Terra 3 Preto E Laranja</t>
+          <t>Tênis Olympikus Corre Trilha 3 Masculino Corrida Original</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1026,14 +1026,14 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://meli.la/2sL3u8E</t>
+          <t>https://meli.la/1oN6h3k</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Tênis Olympikus Corre Trilha 3 Masculino Corrida Original</t>
+          <t>Tênis Masculino Gel-sonoma 8 Verde Asics</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1043,48 +1043,48 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://meli.la/1oN6h3k</t>
+          <t>https://meli.la/16RtefK</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Tênis Masculino Gel-sonoma 8 Verde Asics</t>
+          <t>2 Pares Meia Poliamida Lupo Corrida Power Anti Bolha Curta</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Tenis</t>
+          <t>Meias</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://meli.la/16RtefK</t>
+          <t>https://meli.la/1Zua3RH</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2 Pares Meia Poliamida Lupo Corrida Power Anti Bolha Curta</t>
+          <t>Kit 3 Camisa Proteção Uv Masculina Segunda Pele Sol</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Meias</t>
+          <t>Roupa Termica</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://meli.la/1Zua3RH</t>
+          <t>https://meli.la/1Q3Dw3A</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Kit 3 Camisa Proteção Uv Masculina Segunda Pele Sol</t>
+          <t>Calça Térmica Masculina Legging Esportiva Com Compressão</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1094,14 +1094,14 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://meli.la/1Q3Dw3A</t>
+          <t>https://meli.la/1juShNY</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Calça Térmica Masculina Legging Esportiva Com Compressão</t>
+          <t>Kit 2 Shorts De Compressão P/ Corrida Masculino Térmica</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1111,48 +1111,48 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://meli.la/1juShNY</t>
+          <t>https://meli.la/2KvtjPk</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Kit 2 Shorts De Compressão P/ Corrida Masculino Térmica</t>
+          <t>Tenis Aquático Antiderrapante Neoprene Branquinha Magazine</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Roupa Termica</t>
+          <t>Tenis</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://meli.la/2KvtjPk</t>
+          <t>https://meli.la/1Yr12sF</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Tenis Aquático Antiderrapante Neoprene Branquinha Magazine</t>
+          <t>Capa De Chuva Poncho Compacto Impermeável Ntk Resistente</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Tenis</t>
+          <t>Capa de Chuva</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://meli.la/1Yr12sF</t>
+          <t>https://meli.la/2zs5kVM</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Capa De Chuva Poncho Compacto Impermeável Ntk Resistente</t>
+          <t>Capa De Chuva Com Capuz Ajustável Multifuncional Resistente</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1162,31 +1162,31 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://meli.la/2zs5kVM</t>
+          <t>https://meli.la/2YXwdi6</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Capa De Chuva Com Capuz Ajustável Multifuncional Resistente</t>
+          <t>Power Bank 50.000 mAh Carregador USB Portátil</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Capa de Chuva</t>
+          <t>Powerbank</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://meli.la/2YXwdi6</t>
+          <t>https://meli.la/139kfzg</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Power Bank 50.000 mAh Carregador USB Portátil</t>
+          <t>Power Bank 10000mAh Carregador Portátil Turbo Bahrein</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1196,14 +1196,14 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://meli.la/139kfzg</t>
+          <t>https://meli.la/2tqG1qc</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Power Bank 10000mAh Carregador Portátil Turbo Bahrein</t>
+          <t>Power Bank Tantsa 20000mAh Turbo USB-C 22,5W Preto</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1212,23 +1212,6 @@
         </is>
       </c>
       <c r="C45" t="inlineStr">
-        <is>
-          <t>https://meli.la/2tqG1qc</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Power Bank Tantsa 20000mAh Turbo USB-C 22,5W Preto</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Powerbank</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
         <is>
           <t>https://meli.la/1VR6Xru</t>
         </is>

</xml_diff>

<commit_message>
Cria categoria Capas de Chuva com 4 produtos e remove duplicados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/links.xlsx
+++ b/data/links.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1135,7 +1135,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Capa De Chuva Poncho Compacto Impermeável Ntk Resistente</t>
+          <t>Capa De Chuva Com Capuz Ajustável Multifuncional Resistente</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1145,31 +1145,31 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://meli.la/2zs5kVM</t>
+          <t>https://meli.la/2YXwdi6</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Capa De Chuva Com Capuz Ajustável Multifuncional Resistente</t>
+          <t>Power Bank 50.000 mAh Carregador USB Portátil</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Capa de Chuva</t>
+          <t>Powerbank</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://meli.la/2YXwdi6</t>
+          <t>https://meli.la/139kfzg</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Power Bank 50.000 mAh Carregador USB Portátil</t>
+          <t>Power Bank 10000mAh Carregador Portátil Turbo Bahrein</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1179,14 +1179,14 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://meli.la/139kfzg</t>
+          <t>https://meli.la/2tqG1qc</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Power Bank 10000mAh Carregador Portátil Turbo Bahrein</t>
+          <t>Power Bank Tantsa 20000mAh Turbo USB-C 22,5W Preto</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1196,24 +1196,58 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://meli.la/2tqG1qc</t>
+          <t>https://meli.la/1VR6Xru</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Power Bank Tantsa 20000mAh Turbo USB-C 22,5W Preto</t>
+          <t>Capa De Chuva Poncho Laranja 100% Impermeável Legendários</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Powerbank</t>
+          <t>Capa de Chuva</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://meli.la/1VR6Xru</t>
+          <t>https://meli.la/1YDBzr4</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Capa De Chuva Poncho Compacto Impermeável NTK Laranja</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Capa de Chuva</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://meli.la/2XGbtNH</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Capa De Chuva Impermeável Profissional Adulto Laranja</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Capa de Chuva</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://meli.la/2aBVF3r</t>
         </is>
       </c>
     </row>

</xml_diff>